<commit_message>
feat: add ranking prediction model and optimize virtual table scrolling
Expose regression-based placement predictions in the detail modal, enrich pipeline records with predictions, and improve master table scroll performance with cached filtering and RAF-throttled rendering.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/yokatlas_sonuclar.xlsx
+++ b/yokatlas_sonuclar.xlsx
@@ -557,7 +557,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Bursa</t>
+          <t>BURSA</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
@@ -614,7 +614,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>İzmir</t>
+          <t>İZMİR</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -671,7 +671,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>İSTANBUL</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -728,7 +728,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Edirne</t>
+          <t>EDİRNE</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -748,12 +748,12 @@
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>240,195</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>216,176 - 264,214</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
@@ -785,7 +785,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Zonguldak</t>
+          <t>ZONGULDAK</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -805,12 +805,12 @@
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>293,590</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>264,231 - 322,949</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
@@ -832,7 +832,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>207500164</t>
+          <t>207500157</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -842,7 +842,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>İSTANBUL</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -852,22 +852,22 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>50,000</t>
+          <t>337,954</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>Sürekli Yükselişte ⬆️</t>
+          <t>Yatay ➡️</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>44,115</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>39,704 - 48,527</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
@@ -889,7 +889,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>210403083</t>
+          <t>210403076</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -899,7 +899,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>İSTANBUL</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -909,7 +909,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>922,642</t>
+          <t>214,849</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
@@ -919,12 +919,12 @@
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>930,442</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>837,398 - 1,023,486</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
@@ -946,7 +946,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>208151379</t>
+          <t>208151372</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -956,7 +956,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>İSTANBUL</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
@@ -966,22 +966,22 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>50,000</t>
+          <t>238,292</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>Sürekli Yükselişte ⬆️</t>
+          <t>Yatay ➡️</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>51,900</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>46,710 - 57,090</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
@@ -1013,7 +1013,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>İzmir</t>
+          <t>İZMİR</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
@@ -1070,7 +1070,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Burdur</t>
+          <t>BURDUR</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
@@ -1117,7 +1117,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>205090569</t>
+          <t>205090562</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -1127,7 +1127,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>İSTANBUL</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
@@ -1137,22 +1137,22 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>50,000</t>
+          <t>166,166</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>Sürekli Yükselişte ⬆️</t>
+          <t>Düşüşte ⬇️</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>51,900</t>
+          <t>141,614</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>46,710 - 57,090</t>
+          <t>127,453 - 155,775</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
@@ -1174,7 +1174,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>107690291</t>
+          <t>107610488</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -1184,7 +1184,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Muğla</t>
+          <t>MUĞLA</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
@@ -1194,22 +1194,22 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>263,356</t>
+          <t>145,548</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>Sürekli Yükselişte ⬆️</t>
+          <t>Düşüşte ⬇️</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>183,924</t>
+          <t>89,367</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>165,532 - 202,316</t>
+          <t>80,430 - 98,304</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
@@ -1241,7 +1241,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Bartın</t>
+          <t>BARTIN</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
@@ -1298,7 +1298,7 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Mersin</t>
+          <t>MERSİN</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
@@ -1355,7 +1355,7 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Niğde</t>
+          <t>NİĞDE</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
@@ -1412,7 +1412,7 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Gümüşhane</t>
+          <t>GÜMÜŞHANE</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
@@ -1469,7 +1469,7 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Iğdır</t>
+          <t>IĞDIR</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
@@ -1526,7 +1526,7 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Kahramanmaraş</t>
+          <t>KAHRAMANMARAŞ</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Kütahya</t>
+          <t>KÜTAHYA</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
@@ -1603,12 +1603,12 @@
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>189,389</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>170,450 - 208,328</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
@@ -1640,7 +1640,7 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Burdur</t>
+          <t>BURDUR</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
@@ -1687,7 +1687,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>300590672</t>
+          <t>112700213</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
@@ -1697,7 +1697,7 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>KKTC</t>
+          <t>SAMSUN</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
@@ -1707,22 +1707,22 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>50,000</t>
+          <t>120,344</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>Sürekli Yükselişte ⬆️</t>
+          <t>Düşüşte ⬇️</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>46,710</t>
+          <t>98,004</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>42,039 - 51,381</t>
+          <t>88,204 - 107,804</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
@@ -1754,7 +1754,7 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Karabük</t>
+          <t>KARABÜK</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
@@ -1801,7 +1801,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>405210132</t>
+          <t>101110581</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
@@ -1811,7 +1811,7 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Kırgızistan</t>
+          <t>ANKARA</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
@@ -1821,7 +1821,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>273,374</t>
+          <t>34,690</t>
         </is>
       </c>
       <c r="G24" s="3" t="inlineStr">
@@ -1831,12 +1831,12 @@
       </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
-          <t>268,770</t>
+          <t>28,034</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>241,893 - 295,647</t>
+          <t>25,231 - 30,837</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
@@ -1868,7 +1868,7 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Kazakistan</t>
+          <t>KARABÜK</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
@@ -1888,12 +1888,12 @@
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>228,016</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>205,214 - 250,818</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
@@ -1913,11 +1913,7 @@
           <t>25</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>300290441</t>
-        </is>
-      </c>
+      <c r="B26" s="2" t="inlineStr"/>
       <c r="C26" s="3" t="inlineStr">
         <is>
           <t>GİRNE AMERİKAN ÜNİVERSİTESİ( Vakıf) - Bilgisayar Mühendisliği</t>
@@ -1935,22 +1931,22 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>298,085</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G26" s="3" t="inlineStr">
         <is>
-          <t>Yatay ➡️</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
         <is>
-          <t>183,531</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>165,178 - 201,884</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
@@ -1972,7 +1968,7 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>300390376</t>
+          <t>101110581</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
@@ -1982,7 +1978,7 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>KKTC</t>
+          <t>ANKARA</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
@@ -1992,22 +1988,22 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>269,629</t>
+          <t>34,690</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>Yatay ➡️</t>
+          <t>Düşüşte ⬇️</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr">
         <is>
-          <t>325,678</t>
+          <t>28,034</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>293,110 - 358,246</t>
+          <t>25,231 - 30,837</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr">
@@ -2039,7 +2035,7 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Bingöl</t>
+          <t>BİNGÖL</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
@@ -2096,7 +2092,7 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Osmaniye</t>
+          <t>OSMANİYE</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
@@ -2153,7 +2149,7 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Şanlıurfa</t>
+          <t>KARABÜK</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
@@ -2173,12 +2169,12 @@
       </c>
       <c r="H30" s="4" t="inlineStr">
         <is>
-          <t>228,016</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>205,214 - 250,818</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
@@ -2210,7 +2206,7 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Adıyaman</t>
+          <t>ADIYAMAN</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
@@ -2267,7 +2263,7 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Erzincan</t>
+          <t>ERZİNCAN</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
@@ -2324,7 +2320,7 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Artvin</t>
+          <t>ARTVİN</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
@@ -2381,7 +2377,7 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Mardin</t>
+          <t>MARDİN</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
@@ -2438,7 +2434,7 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Kahramanmaraş</t>
+          <t>KAHRAMANMARAŞ</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
@@ -2495,7 +2491,7 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Malatya</t>
+          <t>MALATYA</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
@@ -2552,7 +2548,7 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Karabük</t>
+          <t>KARABÜK</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
@@ -2572,12 +2568,12 @@
       </c>
       <c r="H37" s="4" t="inlineStr">
         <is>
-          <t>228,016</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>205,214 - 250,818</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr">
@@ -2609,7 +2605,7 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Tokat</t>
+          <t>TOKAT</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
@@ -2666,7 +2662,7 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Çankırı</t>
+          <t>ÇANKIRI</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
@@ -2723,7 +2719,7 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Gaziantep</t>
+          <t>GAZİANTEP</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr">
@@ -2780,7 +2776,7 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Hatay</t>
+          <t>HATAY</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
@@ -2837,7 +2833,7 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Kırşehir</t>
+          <t>KIRŞEHİR</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr">
@@ -2894,7 +2890,7 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>Niğde</t>
+          <t>NİĞDE</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
@@ -2951,7 +2947,7 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Giresun</t>
+          <t>GİRESUN</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr">
@@ -3008,7 +3004,7 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>Rize</t>
+          <t>RİZE</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
@@ -3065,7 +3061,7 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Kastamonu</t>
+          <t>KASTAMONU</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr">
@@ -3122,7 +3118,7 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>Bartın</t>
+          <t>BARTIN</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
@@ -3179,7 +3175,7 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Amasya</t>
+          <t>AMASYA</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr">
@@ -3236,7 +3232,7 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>Kayseri</t>
+          <t>KAYSERİ</t>
         </is>
       </c>
       <c r="E49" s="3" t="inlineStr">
@@ -3256,12 +3252,12 @@
       </c>
       <c r="H49" s="4" t="inlineStr">
         <is>
-          <t>192,100</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I49" s="2" t="inlineStr">
         <is>
-          <t>172,890 - 211,310</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J49" s="2" t="inlineStr">
@@ -3293,7 +3289,7 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Amasya</t>
+          <t>AMASYA</t>
         </is>
       </c>
       <c r="E50" s="3" t="inlineStr">
@@ -3313,12 +3309,12 @@
       </c>
       <c r="H50" s="4" t="inlineStr">
         <is>
-          <t>255,588</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>230,029 - 281,147</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J50" s="2" t="inlineStr">
@@ -3350,7 +3346,7 @@
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>İzmir</t>
+          <t>DÜZCE</t>
         </is>
       </c>
       <c r="E51" s="3" t="inlineStr">
@@ -3397,7 +3393,7 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>103490652</t>
+          <t>103490547</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
@@ -3407,7 +3403,7 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>İzmir</t>
+          <t>İZMİR</t>
         </is>
       </c>
       <c r="E52" s="3" t="inlineStr">
@@ -3417,22 +3413,22 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>50,000</t>
+          <t>350,901</t>
         </is>
       </c>
       <c r="G52" s="3" t="inlineStr">
         <is>
-          <t>Sürekli Yükselişte ⬆️</t>
+          <t>Hafif Yükseliş ↗️</t>
         </is>
       </c>
       <c r="H52" s="4" t="inlineStr">
         <is>
-          <t>44,115</t>
+          <t>395,997</t>
         </is>
       </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t>39,704 - 48,527</t>
+          <t>356,397 - 435,597</t>
         </is>
       </c>
       <c r="J52" s="2" t="inlineStr">
@@ -3464,7 +3460,7 @@
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>İzmir</t>
+          <t>İZMİR</t>
         </is>
       </c>
       <c r="E53" s="3" t="inlineStr">
@@ -3521,7 +3517,7 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>İzmir</t>
+          <t>İZMİR</t>
         </is>
       </c>
       <c r="E54" s="3" t="inlineStr">
@@ -3578,7 +3574,7 @@
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>İzmir</t>
+          <t>DÜZCE</t>
         </is>
       </c>
       <c r="E55" s="3" t="inlineStr">
@@ -3635,7 +3631,7 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>Bursa</t>
+          <t>BURSA</t>
         </is>
       </c>
       <c r="E56" s="3" t="inlineStr">
@@ -3692,7 +3688,7 @@
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>Bursa</t>
+          <t>BURSA</t>
         </is>
       </c>
       <c r="E57" s="3" t="inlineStr">
@@ -3749,7 +3745,7 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>Bursa</t>
+          <t>BURSA</t>
         </is>
       </c>
       <c r="E58" s="3" t="inlineStr">
@@ -3806,7 +3802,7 @@
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>Bursa</t>
+          <t>BURSA</t>
         </is>
       </c>
       <c r="E59" s="3" t="inlineStr">
@@ -3863,7 +3859,7 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>Bursa</t>
+          <t>BURSA</t>
         </is>
       </c>
       <c r="E60" s="3" t="inlineStr">
@@ -3920,7 +3916,7 @@
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>Bursa</t>
+          <t>BURSA</t>
         </is>
       </c>
       <c r="E61" s="3" t="inlineStr">
@@ -3977,7 +3973,7 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>İzmir</t>
+          <t>İZMİR</t>
         </is>
       </c>
       <c r="E62" s="3" t="inlineStr">
@@ -4034,7 +4030,7 @@
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>İzmir</t>
+          <t>İZMİR</t>
         </is>
       </c>
       <c r="E63" s="3" t="inlineStr">
@@ -4081,7 +4077,7 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>103150732</t>
+          <t>103150617</t>
         </is>
       </c>
       <c r="C64" s="3" t="inlineStr">
@@ -4091,7 +4087,7 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>İzmir</t>
+          <t>İZMİR</t>
         </is>
       </c>
       <c r="E64" s="3" t="inlineStr">
@@ -4101,7 +4097,7 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>1,049,990</t>
+          <t>283,913</t>
         </is>
       </c>
       <c r="G64" s="3" t="inlineStr">
@@ -4111,12 +4107,12 @@
       </c>
       <c r="H64" s="4" t="inlineStr">
         <is>
-          <t>1,382,511</t>
+          <t>328,896</t>
         </is>
       </c>
       <c r="I64" s="2" t="inlineStr">
         <is>
-          <t>1,244,260 - 1,520,762</t>
+          <t>296,006 - 361,786</t>
         </is>
       </c>
       <c r="J64" s="2" t="inlineStr">
@@ -4138,7 +4134,7 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>103150705</t>
+          <t>103150335</t>
         </is>
       </c>
       <c r="C65" s="3" t="inlineStr">
@@ -4148,7 +4144,7 @@
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>İzmir</t>
+          <t>İZMİR</t>
         </is>
       </c>
       <c r="E65" s="3" t="inlineStr">
@@ -4158,7 +4154,7 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>552,515</t>
+          <t>304,014</t>
         </is>
       </c>
       <c r="G65" s="3" t="inlineStr">
@@ -4168,12 +4164,12 @@
       </c>
       <c r="H65" s="4" t="inlineStr">
         <is>
-          <t>485,760</t>
+          <t>306,416</t>
         </is>
       </c>
       <c r="I65" s="2" t="inlineStr">
         <is>
-          <t>437,184 - 534,336</t>
+          <t>275,774 - 337,058</t>
         </is>
       </c>
       <c r="J65" s="2" t="inlineStr">
@@ -4205,7 +4201,7 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>İzmir</t>
+          <t>İZMİR</t>
         </is>
       </c>
       <c r="E66" s="3" t="inlineStr">
@@ -4262,7 +4258,7 @@
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>İzmir</t>
+          <t>İZMİR</t>
         </is>
       </c>
       <c r="E67" s="3" t="inlineStr">
@@ -4309,7 +4305,7 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>100751663</t>
+          <t>100751309</t>
         </is>
       </c>
       <c r="C68" s="3" t="inlineStr">
@@ -4319,7 +4315,7 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>Antalya</t>
+          <t>ANTALYA</t>
         </is>
       </c>
       <c r="E68" s="3" t="inlineStr">
@@ -4329,22 +4325,22 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>1,486,662</t>
+          <t>253,416</t>
         </is>
       </c>
       <c r="G68" s="3" t="inlineStr">
         <is>
-          <t>Düşüşte ⬇️</t>
+          <t>Sürekli Yükselişte ⬆️</t>
         </is>
       </c>
       <c r="H68" s="4" t="inlineStr">
         <is>
-          <t>1,153,508</t>
+          <t>281,897</t>
         </is>
       </c>
       <c r="I68" s="2" t="inlineStr">
         <is>
-          <t>1,038,157 - 1,268,859</t>
+          <t>253,707 - 310,087</t>
         </is>
       </c>
       <c r="J68" s="2" t="inlineStr">
@@ -4376,7 +4372,7 @@
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>Antalya</t>
+          <t>ANTALYA</t>
         </is>
       </c>
       <c r="E69" s="3" t="inlineStr">
@@ -4423,7 +4419,7 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>100751354</t>
+          <t>210300486</t>
         </is>
       </c>
       <c r="C70" s="3" t="inlineStr">
@@ -4433,7 +4429,7 @@
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>Antalya</t>
+          <t>İSTANBUL</t>
         </is>
       </c>
       <c r="E70" s="3" t="inlineStr">
@@ -4443,7 +4439,7 @@
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>318,684</t>
+          <t>551,792</t>
         </is>
       </c>
       <c r="G70" s="3" t="inlineStr">
@@ -4453,12 +4449,12 @@
       </c>
       <c r="H70" s="4" t="inlineStr">
         <is>
-          <t>378,462</t>
+          <t>571,474</t>
         </is>
       </c>
       <c r="I70" s="2" t="inlineStr">
         <is>
-          <t>340,616 - 416,308</t>
+          <t>514,327 - 628,621</t>
         </is>
       </c>
       <c r="J70" s="2" t="inlineStr">
@@ -4490,7 +4486,7 @@
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>Antalya</t>
+          <t>ANTALYA</t>
         </is>
       </c>
       <c r="E71" s="3" t="inlineStr">
@@ -4510,12 +4506,12 @@
       </c>
       <c r="H71" s="4" t="inlineStr">
         <is>
-          <t>596,699</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I71" s="2" t="inlineStr">
         <is>
-          <t>537,029 - 656,369</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J71" s="2" t="inlineStr">
@@ -4547,7 +4543,7 @@
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>Antalya</t>
+          <t>DÜZCE</t>
         </is>
       </c>
       <c r="E72" s="3" t="inlineStr">
@@ -4567,12 +4563,12 @@
       </c>
       <c r="H72" s="4" t="inlineStr">
         <is>
-          <t>771,370</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I72" s="2" t="inlineStr">
         <is>
-          <t>694,233 - 848,507</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J72" s="2" t="inlineStr">
@@ -4604,7 +4600,7 @@
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>Eskişehir</t>
+          <t>ESKİŞEHİR</t>
         </is>
       </c>
       <c r="E73" s="3" t="inlineStr">
@@ -4624,12 +4620,12 @@
       </c>
       <c r="H73" s="4" t="inlineStr">
         <is>
-          <t>231,556</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I73" s="2" t="inlineStr">
         <is>
-          <t>208,400 - 254,712</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J73" s="2" t="inlineStr">
@@ -4661,7 +4657,7 @@
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>Eskişehir</t>
+          <t>ESKİŞEHİR</t>
         </is>
       </c>
       <c r="E74" s="3" t="inlineStr">
@@ -4718,7 +4714,7 @@
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>Eskişehir</t>
+          <t>ESKİŞEHİR</t>
         </is>
       </c>
       <c r="E75" s="3" t="inlineStr">
@@ -4775,7 +4771,7 @@
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>Eskişehir</t>
+          <t>ESKİŞEHİR</t>
         </is>
       </c>
       <c r="E76" s="3" t="inlineStr">
@@ -4832,7 +4828,7 @@
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>Eskişehir</t>
+          <t>ESKİŞEHİR</t>
         </is>
       </c>
       <c r="E77" s="3" t="inlineStr">
@@ -4889,7 +4885,7 @@
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>Eskişehir</t>
+          <t>ESKİŞEHİR</t>
         </is>
       </c>
       <c r="E78" s="3" t="inlineStr">
@@ -4946,7 +4942,7 @@
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>Eskişehir</t>
+          <t>ESKİŞEHİR</t>
         </is>
       </c>
       <c r="E79" s="3" t="inlineStr">
@@ -5003,7 +4999,7 @@
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>KARABÜK</t>
         </is>
       </c>
       <c r="E80" s="3" t="inlineStr">
@@ -5060,7 +5056,7 @@
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>KARABÜK</t>
         </is>
       </c>
       <c r="E81" s="3" t="inlineStr">
@@ -5117,7 +5113,7 @@
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>ANKARA</t>
         </is>
       </c>
       <c r="E82" s="3" t="inlineStr">
@@ -5164,7 +5160,7 @@
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>107450356</t>
+          <t>109890128</t>
         </is>
       </c>
       <c r="C83" s="3" t="inlineStr">
@@ -5174,7 +5170,7 @@
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>UŞAK</t>
         </is>
       </c>
       <c r="E83" s="3" t="inlineStr">
@@ -5184,7 +5180,7 @@
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>684,068</t>
+          <t>975,711</t>
         </is>
       </c>
       <c r="G83" s="3" t="inlineStr">
@@ -5194,12 +5190,12 @@
       </c>
       <c r="H83" s="4" t="inlineStr">
         <is>
-          <t>633,105</t>
+          <t>1,242,497</t>
         </is>
       </c>
       <c r="I83" s="2" t="inlineStr">
         <is>
-          <t>569,794 - 696,416</t>
+          <t>1,118,247 - 1,366,747</t>
         </is>
       </c>
       <c r="J83" s="2" t="inlineStr">
@@ -5221,7 +5217,7 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>107290432</t>
+          <t>107250437</t>
         </is>
       </c>
       <c r="C84" s="3" t="inlineStr">
@@ -5231,7 +5227,7 @@
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>İSTANBUL</t>
         </is>
       </c>
       <c r="E84" s="3" t="inlineStr">
@@ -5241,7 +5237,7 @@
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>883,899</t>
+          <t>309,714</t>
         </is>
       </c>
       <c r="G84" s="3" t="inlineStr">
@@ -5251,12 +5247,12 @@
       </c>
       <c r="H84" s="4" t="inlineStr">
         <is>
-          <t>611,928</t>
+          <t>383,883</t>
         </is>
       </c>
       <c r="I84" s="2" t="inlineStr">
         <is>
-          <t>550,735 - 673,121</t>
+          <t>345,495 - 422,271</t>
         </is>
       </c>
       <c r="J84" s="2" t="inlineStr">
@@ -5288,7 +5284,7 @@
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>HAKKARİ</t>
         </is>
       </c>
       <c r="E85" s="3" t="inlineStr">
@@ -5345,7 +5341,7 @@
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>İSTANBUL</t>
         </is>
       </c>
       <c r="E86" s="3" t="inlineStr">
@@ -5402,7 +5398,7 @@
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>ANKARA</t>
         </is>
       </c>
       <c r="E87" s="3" t="inlineStr">
@@ -5459,7 +5455,7 @@
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>KARABÜK</t>
         </is>
       </c>
       <c r="E88" s="3" t="inlineStr">
@@ -5516,7 +5512,7 @@
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>İSTANBUL</t>
         </is>
       </c>
       <c r="E89" s="3" t="inlineStr">
@@ -5573,7 +5569,7 @@
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>İSTANBUL</t>
         </is>
       </c>
       <c r="E90" s="3" t="inlineStr">
@@ -5630,7 +5626,7 @@
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>İSTANBUL</t>
         </is>
       </c>
       <c r="E91" s="3" t="inlineStr">
@@ -5687,7 +5683,7 @@
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>İSTANBUL</t>
         </is>
       </c>
       <c r="E92" s="3" t="inlineStr">
@@ -5744,7 +5740,7 @@
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>İSTANBUL</t>
         </is>
       </c>
       <c r="E93" s="3" t="inlineStr">
@@ -5801,7 +5797,7 @@
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>İSTANBUL</t>
         </is>
       </c>
       <c r="E94" s="3" t="inlineStr">
@@ -5858,7 +5854,7 @@
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>İSTANBUL</t>
         </is>
       </c>
       <c r="E95" s="3" t="inlineStr">
@@ -5915,7 +5911,7 @@
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>İSTANBUL</t>
         </is>
       </c>
       <c r="E96" s="3" t="inlineStr">
@@ -5972,7 +5968,7 @@
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>İSTANBUL</t>
         </is>
       </c>
       <c r="E97" s="3" t="inlineStr">

</xml_diff>